<commit_message>
docs(vestventures): runda scade la 150k €, deck-ul de 12 slide-uri, fără procentele de proprietate
Modelul refăcut pe un plan strâns: 24 de luni de runway pe planul de bază,
16 fără venituri, seed la 100 de clienți în luna 20. Planul, cap table-ul,
roadmap-ul, formularul și README-ul preiau cifrele din cifre.json. Deck-ul
are un singur mesaj pe slide; detaliile de capital rămân în cap-table.pdf.
Sincronizat pe Drive în aceleași fișiere.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vestventures/cap-table.xlsx
+++ b/vestventures/cap-table.xlsx
@@ -210,7 +210,7 @@
     <t xml:space="preserve">Years until conversion</t>
   </si>
   <si>
-    <t xml:space="preserve">ILLUSTRATIVE (seed ~18 months after close)</t>
+    <t xml:space="preserve">ILLUSTRATIVE (seed ~24 months after close: 100-customer trigger + raise)</t>
   </si>
   <si>
     <t xml:space="preserve">Amount converting (EUR)</t>
@@ -736,7 +736,7 @@
         <v>10</v>
       </c>
       <c r="B8" s="7" t="n">
-        <v>200000</v>
+        <v>135000</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -754,7 +754,7 @@
         <v>12</v>
       </c>
       <c r="B9" s="7" t="n">
-        <v>50000</v>
+        <v>15000</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
@@ -889,7 +889,7 @@
       </c>
       <c r="B17" s="11" t="n">
         <f aca="false">B8+B9</f>
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -906,7 +906,7 @@
       </c>
       <c r="B18" s="11" t="n">
         <f aca="false">B10+B17</f>
-        <v>1500000</v>
+        <v>1400000</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -923,7 +923,7 @@
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">B17/B18</f>
-        <v>0.166666666666667</v>
+        <v>0.107142857142857</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -940,7 +940,7 @@
       </c>
       <c r="B20" s="13" t="n">
         <f aca="false">B5/(1-B19-B11)</f>
-        <v>13636.3636363636</v>
+        <v>12612.6126126126</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -957,7 +957,7 @@
       </c>
       <c r="B21" s="14" t="n">
         <f aca="false">B10/(B5+B11*B20)</f>
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B24" s="13" t="n">
         <f aca="false">B20/(1-B23-B14)</f>
-        <v>17045.4545454545</v>
+        <v>15765.7657657658</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
@@ -1025,7 +1025,7 @@
       </c>
       <c r="B25" s="14" t="n">
         <f aca="false">B13/(B20+B14*B24)</f>
-        <v>293.333333333333</v>
+        <v>317.142857142857</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="E29" s="12" t="n">
         <f aca="false">D29/$D$35</f>
-        <v>0.374</v>
+        <v>0.404357142857143</v>
       </c>
       <c r="F29" s="13" t="n">
         <f aca="false">D29</f>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="G29" s="12" t="n">
         <f aca="false">F29/$F$35</f>
-        <v>0.2992</v>
+        <v>0.323485714285714</v>
       </c>
       <c r="H29" s="11" t="n">
         <v>0</v>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="E30" s="12" t="n">
         <f aca="false">D30/$D$35</f>
-        <v>0.359333333333333</v>
+        <v>0.3885</v>
       </c>
       <c r="F30" s="13" t="n">
         <f aca="false">D30</f>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="G30" s="12" t="n">
         <f aca="false">F30/$F$35</f>
-        <v>0.287466666666667</v>
+        <v>0.3108</v>
       </c>
       <c r="H30" s="11" t="n">
         <v>0</v>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="D31" s="13" t="n">
         <f aca="false">B11*B20</f>
-        <v>1363.63636363636</v>
+        <v>1261.26126126126</v>
       </c>
       <c r="E31" s="12" t="n">
         <f aca="false">D31/$D$35</f>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="F31" s="13" t="n">
         <f aca="false">D31+B14*B24</f>
-        <v>1363.63636363636</v>
+        <v>1261.26126126126</v>
       </c>
       <c r="G31" s="12" t="n">
         <f aca="false">F31/$F$35</f>
@@ -1202,23 +1202,23 @@
       </c>
       <c r="D32" s="13" t="n">
         <f aca="false">B8/B21</f>
-        <v>1818.18181818182</v>
+        <v>1216.21621621622</v>
       </c>
       <c r="E32" s="12" t="n">
         <f aca="false">D32/$D$35</f>
-        <v>0.133333333333333</v>
+        <v>0.0964285714285714</v>
       </c>
       <c r="F32" s="13" t="n">
         <f aca="false">D32</f>
-        <v>1818.18181818182</v>
+        <v>1216.21621621622</v>
       </c>
       <c r="G32" s="12" t="n">
         <f aca="false">F32/$F$35</f>
-        <v>0.106666666666667</v>
+        <v>0.0771428571428572</v>
       </c>
       <c r="H32" s="11" t="n">
         <f aca="false">B8</f>
-        <v>200000</v>
+        <v>135000</v>
       </c>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
@@ -1236,23 +1236,23 @@
       </c>
       <c r="D33" s="13" t="n">
         <f aca="false">B9/B21</f>
-        <v>454.545454545455</v>
+        <v>135.135135135135</v>
       </c>
       <c r="E33" s="12" t="n">
         <f aca="false">D33/$D$35</f>
-        <v>0.0333333333333333</v>
+        <v>0.0107142857142857</v>
       </c>
       <c r="F33" s="13" t="n">
         <f aca="false">D33</f>
-        <v>454.545454545455</v>
+        <v>135.135135135135</v>
       </c>
       <c r="G33" s="12" t="n">
         <f aca="false">F33/$F$35</f>
-        <v>0.0266666666666667</v>
+        <v>0.00857142857142857</v>
       </c>
       <c r="H33" s="11" t="n">
         <f aca="false">B9</f>
-        <v>50000</v>
+        <v>15000</v>
       </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="F34" s="13" t="n">
         <f aca="false">B12/B25</f>
-        <v>3409.09090909091</v>
+        <v>3153.15315315315</v>
       </c>
       <c r="G34" s="12" t="n">
         <f aca="false">F34/$F$35</f>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D35" s="15" t="n">
         <f aca="false">SUM(D29:D34)</f>
-        <v>13636.3636363636</v>
+        <v>12612.6126126126</v>
       </c>
       <c r="E35" s="16" t="n">
         <f aca="false">SUM(E29:E34)</f>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="F35" s="15" t="n">
         <f aca="false">SUM(F29:F34)</f>
-        <v>17045.4545454545</v>
+        <v>15765.7657657658</v>
       </c>
       <c r="G35" s="16" t="n">
         <f aca="false">SUM(G29:G34)</f>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="H35" s="17" t="n">
         <f aca="false">SUM(H29:H34)</f>
-        <v>1250000</v>
+        <v>1150000</v>
       </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
@@ -1337,12 +1337,12 @@
       <c r="D36" s="2"/>
       <c r="E36" s="12" t="n">
         <f aca="false">E29+E30</f>
-        <v>0.733333333333333</v>
+        <v>0.792857142857143</v>
       </c>
       <c r="F36" s="2"/>
       <c r="G36" s="12" t="n">
         <f aca="false">G29+G30</f>
-        <v>0.586666666666667</v>
+        <v>0.634285714285714</v>
       </c>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
@@ -1356,7 +1356,7 @@
       <c r="C37" s="2"/>
       <c r="D37" s="11" t="n">
         <f aca="false">D35*B21</f>
-        <v>1500000</v>
+        <v>1400000</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" s="11" t="n">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="B4" s="18" t="n">
         <f aca="false">'Cap table'!B17</f>
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>54</v>
@@ -1462,7 +1462,7 @@
         <v>61</v>
       </c>
       <c r="B8" s="19" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>62</v>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="B9" s="11" t="n">
         <f aca="false">B4*(1+B7*B8)</f>
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="C9" s="3"/>
     </row>
@@ -1484,7 +1484,7 @@
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">'Cap table'!B5+'Cap table'!D31</f>
-        <v>11363.6363636364</v>
+        <v>11261.2612612613</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>65</v>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="B11" s="14" t="n">
         <f aca="false">B5/B10</f>
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>67</v>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="B12" s="21" t="n">
         <f aca="false">'Cap table'!B13/B10</f>
-        <v>352</v>
+        <v>355.2</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>69</v>
@@ -1520,7 +1520,7 @@
       </c>
       <c r="B13" s="14" t="n">
         <f aca="false">B12*(1-B6)</f>
-        <v>281.6</v>
+        <v>284.16</v>
       </c>
       <c r="C13" s="3"/>
     </row>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="B14" s="14" t="n">
         <f aca="false">MIN(B11,B13)</f>
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C14" s="3"/>
     </row>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="B15" s="13" t="n">
         <f aca="false">B9/B14</f>
-        <v>2272.72727272727</v>
+        <v>1351.35135135135</v>
       </c>
       <c r="C15" s="3"/>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="B16" s="12" t="n">
         <f aca="false">B15/(B10+B15)</f>
-        <v>0.166666666666667</v>
+        <v>0.107142857142857</v>
       </c>
       <c r="C16" s="3"/>
     </row>
@@ -1570,7 +1570,7 @@
       </c>
       <c r="B18" s="20" t="n">
         <f aca="false">B17/('Cap table'!B13/(B10+B15))</f>
-        <v>3409.09090909091</v>
+        <v>3153.15315315315</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>76</v>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="B19" s="13" t="n">
         <f aca="false">B10+B15+B18</f>
-        <v>17045.4545454545</v>
+        <v>15765.7657657658</v>
       </c>
       <c r="C19" s="3"/>
     </row>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="B20" s="22" t="n">
         <f aca="false">('Cap table'!B5)/B19</f>
-        <v>0.586666666666667</v>
+        <v>0.634285714285714</v>
       </c>
       <c r="C20" s="3"/>
     </row>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="B21" s="22" t="n">
         <f aca="false">'Cap table'!G36</f>
-        <v>0.586666666666667</v>
+        <v>0.634285714285714</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>80</v>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">B15/B19</f>
-        <v>0.133333333333333</v>
+        <v>0.0857142857142857</v>
       </c>
       <c r="C22" s="3"/>
     </row>

</xml_diff>